<commit_message>
Fix employee records table and add PF/ESIC contribution columns
</commit_message>
<xml_diff>
--- a/uploads/Book1.xlsx
+++ b/uploads/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0602134B-ED92-44F9-B9A2-53F20381BDC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{887BEA00-D700-4E40-8774-F3D5B095E1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F902CF28-21A3-4E3F-905C-D7D2FE32720D}"/>
   </bookViews>
@@ -25,52 +25,114 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UAN </t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMPLOYEE </t>
-  </si>
-  <si>
-    <t>BASIC</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+  <si>
+    <t>Prince</t>
+  </si>
+  <si>
+    <t>100025689520</t>
+  </si>
+  <si>
+    <t>OP Manager</t>
+  </si>
+  <si>
+    <t>SBI765890</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Employee Code</t>
+  </si>
+  <si>
+    <t>UAN</t>
+  </si>
+  <si>
+    <t>ESIC Number</t>
+  </si>
+  <si>
+    <t>Designation</t>
+  </si>
+  <si>
+    <t>Working Days</t>
+  </si>
+  <si>
+    <t>PF Wages</t>
+  </si>
+  <si>
+    <t>PF Contribution</t>
+  </si>
+  <si>
+    <t>ESIC Contribution</t>
+  </si>
+  <si>
+    <t>Gross</t>
+  </si>
+  <si>
+    <t>Deductions</t>
+  </si>
+  <si>
+    <t>Net Salary</t>
+  </si>
+  <si>
+    <t>OT</t>
+  </si>
+  <si>
+    <t>Bank Transfer Reference</t>
+  </si>
+  <si>
+    <t>Bonus Detail</t>
+  </si>
+  <si>
+    <t>Bonus Paid Date</t>
+  </si>
+  <si>
+    <t>Leave Encashment</t>
+  </si>
+  <si>
+    <t>Fine Detail</t>
+  </si>
+  <si>
+    <t>Damage &amp; Loss Detail</t>
+  </si>
+  <si>
+    <t>rishi</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
   </si>
   <si>
     <t>HRA</t>
   </si>
   <si>
-    <t>OTHER ALL</t>
-  </si>
-  <si>
-    <t>WD</t>
-  </si>
-  <si>
-    <t>PF</t>
-  </si>
-  <si>
-    <t>ESIC</t>
-  </si>
-  <si>
-    <t>GROSS</t>
-  </si>
-  <si>
-    <t>NET</t>
+    <t>Advance Salary</t>
+  </si>
+  <si>
+    <t>Leave Record</t>
+  </si>
+  <si>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>Any Other Allowance</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -93,8 +155,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -409,45 +476,259 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F20E515-E6C7-4374-AAC8-E747D51DE363}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.6640625" customWidth="1"/>
+    <col min="13" max="13" width="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:25" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y1" s="2"/>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>10011</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D2">
+        <v>11345690</v>
+      </c>
+      <c r="E2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F2">
+        <v>28</v>
+      </c>
+      <c r="G2">
+        <v>15000</v>
+      </c>
+      <c r="H2">
+        <v>5000</v>
+      </c>
+      <c r="I2">
+        <v>5000</v>
+      </c>
+      <c r="J2">
+        <v>15000</v>
+      </c>
+      <c r="K2">
+        <v>1800</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>25000</v>
+      </c>
+      <c r="N2">
+        <v>1800</v>
+      </c>
+      <c r="O2">
+        <v>23200</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
+      <c r="U2">
+        <v>2</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>10011</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>11345690</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>28</v>
+      </c>
+      <c r="G3">
+        <v>15000</v>
+      </c>
+      <c r="H3">
+        <v>5000</v>
+      </c>
+      <c r="I3">
+        <v>5000</v>
+      </c>
+      <c r="J3">
+        <v>15000</v>
+      </c>
+      <c r="K3">
+        <v>1800</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>25000</v>
+      </c>
+      <c r="N3">
+        <v>1800</v>
+      </c>
+      <c r="O3">
+        <v>23200</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3" t="s">
+        <v>3</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s">
+        <v>4</v>
+      </c>
+      <c r="U3">
+        <v>2</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>